<commit_message>
Added Details to original DB
</commit_message>
<xml_diff>
--- a/data/seed/student_combined_data.xlsx
+++ b/data/seed/student_combined_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2d704ffe42a61a63/Desktop/Attendance-Companion/data/seed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{88B02031-66B0-4BA6-940A-5C1B3CF45E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D397EB1-44FE-47B8-8D90-05B8F95F55A3}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{88B02031-66B0-4BA6-940A-5C1B3CF45E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5515865-E0B9-4717-A9B6-D3938FCCCA65}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="403">
   <si>
     <t>Combined Student Data — Roll No, Admission No, Name, Section</t>
   </si>
@@ -826,9 +826,6 @@
     <t>2025B01011381</t>
   </si>
   <si>
-    <t>Phone no.</t>
-  </si>
-  <si>
     <t>SUNDARAM TIWARI</t>
   </si>
   <si>
@@ -836,13 +833,410 @@
   </si>
   <si>
     <t>2025B01010048</t>
+  </si>
+  <si>
+    <t>sonali.25b01010503@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sonam.25b01010133@abes.ac.in</t>
+  </si>
+  <si>
+    <t>soumya,25b01011289@abes.ac.in</t>
+  </si>
+  <si>
+    <t>soyanshu.25b01010140@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sparsh.25b01011238@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sri.25b01011179@abes.ac.in</t>
+  </si>
+  <si>
+    <t>srijan.25b01011350@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sudhanshu.25b01010704@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sujeet.25b01010824@gmail.com</t>
+  </si>
+  <si>
+    <t>sundaram.25b01011126@abes.ac.in</t>
+  </si>
+  <si>
+    <t>suryansh.25b01010185@abes.ac.in</t>
+  </si>
+  <si>
+    <t>suryansh.25b01010610@abes.ac.in</t>
+  </si>
+  <si>
+    <t>swarnim.25b01010005@abes.ac.in</t>
+  </si>
+  <si>
+    <t>swastika.25b01010026@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tanishka.25b01010168@abes.ac.in</t>
+  </si>
+  <si>
+    <t>taniya.25b01011017@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tannu.25b01010714@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tarang.25b01010474@abes.ac.in</t>
+  </si>
+  <si>
+    <t>toshit.25b01010754@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tripti.25b01010781@abes.ac.in</t>
+  </si>
+  <si>
+    <t>trishant.250b01011161@abes.ac.in</t>
+  </si>
+  <si>
+    <t>trishya.25b01010568@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tulsi.25b01011130@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01010580@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01010566@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01010936@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01010404@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01010753@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01010446@abes.ac.in</t>
+  </si>
+  <si>
+    <t>uday.25b01011248@abes.ac.in</t>
+  </si>
+  <si>
+    <t>uday.25b01011342@abes.ac.in</t>
+  </si>
+  <si>
+    <t>ujjwal.25b01010991@abes.ac.in</t>
+  </si>
+  <si>
+    <t>ujjwal.25b01010477@abes.ac.in</t>
+  </si>
+  <si>
+    <t>urfa.25b01011320@abes.ac.in</t>
+  </si>
+  <si>
+    <t>utkarsh.25b01010990@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaibhav.25b01010226@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaibhavi.25b01011274@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaishnavi.25b01010224@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaishnavi.25b01010988@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaishnavi.25b01011148@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01011072@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01010197@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vanshika.25b01010202@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vardaan.25b01010007@abes.ac.in</t>
+  </si>
+  <si>
+    <t>varun.25b01011044@abes.ac.in</t>
+  </si>
+  <si>
+    <t>varun.25b01010807@abes.ac.in</t>
+  </si>
+  <si>
+    <t>venkatesh.25b01010015@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vidhan.25b01010931@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vikal.25b01010328@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vikash.25b01010179@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vinay.25b01010232@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vindhyavasini.25b01010521@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vishal.25b01010471@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vivek.25b01010928@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vivek.25b01010914@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vranda.25b01010895@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01010533@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01011117@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01010287@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01010048@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yashasvi.25b01010250@abes.ac.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yashika.25b01010734@abes.ac.in
+</t>
+  </si>
+  <si>
+    <t>yashraj.25b01010249@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yuvraj.25b01010899@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yuvraj.25b01011270@abes.ac.in</t>
+  </si>
+  <si>
+    <t>soumya.25b01010067@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sudiksha.25b01010972@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sumit.25b01011176@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sumit.25b01010627@abes.ac.in</t>
+  </si>
+  <si>
+    <t>sunishtha.25b01010652@abes.ac.in</t>
+  </si>
+  <si>
+    <t>suraj.25b01010440@abes.ac.in</t>
+  </si>
+  <si>
+    <t>surya.25b01010352@abes.ac.in</t>
+  </si>
+  <si>
+    <t>suryansh.25b01010439@abes.ac.in</t>
+  </si>
+  <si>
+    <t>suyash.25b01010013@abes.ac.in</t>
+  </si>
+  <si>
+    <t>swastik.25b01010038@abes.ac.in</t>
+  </si>
+  <si>
+    <t>swastika.25b01010217@abes.ac.in</t>
+  </si>
+  <si>
+    <t>swayam.25b01011076@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tanish.25b01010028@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tanishka.25b01010744@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tanmay.25b01010606@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tarang.25b01010244@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tarun.25b01010604@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tarun.25b01010853@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tejbahadur.25b01010412@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tripti.25b01010953@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushar.25b01011230@abes.ac.in</t>
+  </si>
+  <si>
+    <t>tushti.25b01010259@abes.ac.in</t>
+  </si>
+  <si>
+    <t>ujjawal.25b01010833@abes.ac.in</t>
+  </si>
+  <si>
+    <t>umang.25b01010438@abes.ac.in</t>
+  </si>
+  <si>
+    <t>utkarsh.25b01010402@abes.ac.in</t>
+  </si>
+  <si>
+    <t>utkarsh.25b01010916@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vadanta.25b01010055@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaibhav.25b01010341@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vaishnavi.25b01010702@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01011396@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01010639@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01010052@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01010101@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vansh.25b01010784@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vanshika.25b01010046@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vanshika.25b01010366@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vanshika.25b01010433@abes.ac.in</t>
+  </si>
+  <si>
+    <t>varshita.25b01011381@abes.ac.in</t>
+  </si>
+  <si>
+    <t>varun.25b01010452@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vatsal.25b01011254@abes.ac.in</t>
+  </si>
+  <si>
+    <t>ved.25b01010793@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vedansh.25b01010505@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vedansh.25b01010728@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vedanshi.25b01010057@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vedant.25b01011278@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vedant.25b01010115@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vijay.25b01010780@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vikash.25b01010127@abes.in</t>
+  </si>
+  <si>
+    <t>vishal.25b01010059@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vishesh.25b01011021@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vishesh.25b01010118@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vivek.25b01011358@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vivek.25b01011116@abes.ac.in</t>
+  </si>
+  <si>
+    <t>vrinda.25b01010896@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yadav.25b01010760@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01010992@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01010619@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01010967@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yash.25b01011258@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yashdeep.25b01010525@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yashika.25b01010838@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yashika.25b01010428@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yatharth.25b01010135@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yogansh.25b01011185@abes.ac.in</t>
+  </si>
+  <si>
+    <t>yug.25b01010206@abes.ac.in</t>
+  </si>
+  <si>
+    <t>mobile</t>
+  </si>
+  <si>
+    <t>email</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -879,6 +1273,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -899,7 +1299,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -922,11 +1322,61 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -948,16 +1398,35 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1262,18 +1731,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="20" style="5" customWidth="1"/>
     <col min="3" max="3" width="34" style="5" customWidth="1"/>
     <col min="4" max="4" width="32.88671875" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="38.33203125" style="17" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1281,8 +1751,9 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F1" s="3"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1295,2492 +1766,2943 @@
       <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
         <v>1</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <v>2503201001175</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="13"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E4" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="10">
+        <v>9211088145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>2</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <v>2503201001177</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="13"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C5" s="10"/>
+      <c r="D5" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="E5" s="18"/>
+      <c r="F5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="21"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
         <v>3</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="10">
         <v>2503201001190</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="13"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E6" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="10">
+        <v>7887075764</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
         <v>4</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <v>2503201001192</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="13"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E7" s="18"/>
+      <c r="F7" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="21"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
         <v>5</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <v>2503201001195</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="13"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E8" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="21"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>6</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <v>2503201001197</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="13"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E9" s="18" t="s">
+        <v>339</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="21"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>7</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="10">
         <v>2503201001199</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="13"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E10" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="21"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>8</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <v>2503201001202</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="13"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E11" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="21"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
         <v>9</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="10">
         <v>2503201001203</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E12" s="18" t="s">
+        <v>342</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="21"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>10</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <v>2503201001206</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="13"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E13" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="10">
+        <v>7017742948</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
         <v>11</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <v>2503201001209</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="13"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E14" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="21"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>12</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <v>2503201001212</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="13"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E15" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="10">
+        <v>9456822664</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
         <v>13</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="10">
         <v>2503201001214</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="13"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E16" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="10">
+        <v>8707820552</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>14</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <v>2503201001215</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="E17" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="13"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E17" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="21"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>15</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="10">
         <v>2503201001220</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="13"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E18" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="21"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>16</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <v>2503201001223</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="13"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E19" s="18" t="s">
+        <v>349</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="21"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="9">
         <v>17</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="10">
         <v>2503201001228</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F20" s="13"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E20" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" s="21"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>18</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <v>2503201001232</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" s="13"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E21" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" s="21"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>19</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="10">
         <v>2503201001233</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F22" s="13"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E22" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" s="21"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>20</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <v>2503201001234</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="E23" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F23" s="13"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E23" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="10">
+        <v>9311348641</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
         <v>21</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="10">
         <v>2503201001236</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F24" s="13"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E24" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G24" s="21"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>22</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="10">
         <v>2503201001239</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" s="13">
-        <v>9971225379</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E25" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" s="21"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="9">
         <v>23</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="10">
         <v>2503201001250</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E26" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="13">
-        <v>6299440012</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E26" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" s="10">
+        <v>9971225379</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="9">
         <v>24</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="10">
         <v>2503201001252</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F27" s="13">
-        <v>7465009880</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E27" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G27" s="10">
+        <v>6299440012</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="9">
         <v>25</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="10">
         <v>2503201001257</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="E28" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F28" s="13">
-        <v>9129971514</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E28" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G28" s="10">
+        <v>7465009880</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="9">
         <v>26</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="10">
         <v>2503201001262</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="E29" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F29" s="13">
-        <v>9528558924</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E29" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" s="10">
+        <v>9129971514</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="9">
         <v>27</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="10">
         <v>2503201001266</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F30" s="13">
-        <v>8707848463</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E30" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="F30" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G30" s="10">
+        <v>9528558924</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="9">
         <v>28</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="10">
         <v>2503201001268</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="E31" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F31" s="13">
-        <v>9711297960</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E31" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G31" s="10">
+        <v>8707848463</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="9">
         <v>29</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="10">
         <v>2503201001271</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F32" s="13">
-        <v>7579888767</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E32" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="F32" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G32" s="10">
+        <v>9711297960</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="9">
         <v>30</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="10">
         <v>2503201001273</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E33" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F33" s="13"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E33" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G33" s="10">
+        <v>7579888767</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="9">
         <v>31</v>
       </c>
-      <c r="B34" s="11">
+      <c r="B34" s="10">
         <v>2503201001279</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="E34" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F34" s="13">
-        <v>8595611145</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E34" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G34" s="21"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="9">
         <v>32</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="10">
         <v>2503201001283</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="E35" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F35" s="13"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E35" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="F35" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" s="10">
+        <v>8595611145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="9">
         <v>33</v>
       </c>
-      <c r="B36" s="11">
+      <c r="B36" s="10">
         <v>2503201001284</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="E36" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F36" s="13"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E36" s="18" t="s">
+        <v>366</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G36" s="10">
+        <v>9719586644</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="9">
         <v>34</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="10">
         <v>2503201001286</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E37" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F37" s="13"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E37" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="F37" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G37" s="10">
+        <v>9411792254</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="9">
         <v>35</v>
       </c>
-      <c r="B38" s="11">
+      <c r="B38" s="10">
         <v>2503201001288</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="E38" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F38" s="13"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E38" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="F38" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="G38" s="10">
+        <v>9068718735</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="9">
         <v>36</v>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="10">
         <v>2503201001290</v>
       </c>
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E39" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F39" s="13"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E39" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="F39" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G39" s="10">
+        <v>9634487600</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="9">
         <v>37</v>
       </c>
-      <c r="B40" s="11">
+      <c r="B40" s="10">
         <v>2503201001293</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="E40" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F40" s="13">
-        <v>6393541228</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E40" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="F40" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G40" s="10">
+        <v>9149131768</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="9">
         <v>38</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="10">
         <v>2503201001295</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="E41" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F41" s="13">
-        <v>8679339293</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E41" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G41" s="10">
+        <v>6393541228</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="9">
         <v>39</v>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="10">
         <v>2503201001296</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="E42" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F42" s="13"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E42" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="F42" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G42" s="21"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="9">
         <v>40</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="10">
         <v>2503201001300</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="E43" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F43" s="13">
-        <v>7827624547</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E43" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="F43" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G43" s="10">
+        <v>8171887507</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="9">
         <v>41</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="10">
         <v>2503201001301</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="E44" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F44" s="13"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E44" s="18" t="s">
+        <v>374</v>
+      </c>
+      <c r="F44" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G44" s="10">
+        <v>7827624547</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="9">
         <v>42</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="10">
         <v>2503201001305</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E45" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F45" s="13"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E45" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G45" s="10">
+        <v>7042557172</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="9">
         <v>43</v>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="10">
         <v>2503201001307</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D46" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E46" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F46" s="13"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E46" s="18" t="s">
+        <v>376</v>
+      </c>
+      <c r="F46" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G46" s="21"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="9">
         <v>44</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="10">
         <v>2503201001308</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="D47" s="10" t="s">
+      <c r="D47" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="E47" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F47" s="13"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E47" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="F47" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G47" s="10">
+        <v>8755796352</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="9">
         <v>45</v>
       </c>
-      <c r="B48" s="11">
+      <c r="B48" s="10">
         <v>2503201001309</v>
       </c>
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="D48" s="10" t="s">
+      <c r="D48" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="E48" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F48" s="13"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E48" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="F48" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G48" s="21"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="9">
         <v>46</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="10">
         <v>2503201001310</v>
       </c>
-      <c r="C49" s="11" t="s">
+      <c r="C49" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="D49" s="10" t="s">
+      <c r="D49" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="E49" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F49" s="13"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E49" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="F49" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G49" s="10">
+        <v>7678662753</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="9">
         <v>47</v>
       </c>
-      <c r="B50" s="11">
+      <c r="B50" s="10">
         <v>2503201001311</v>
       </c>
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="D50" s="10" t="s">
+      <c r="D50" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="E50" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F50" s="13"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E50" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="F50" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G50" s="10">
+        <v>9211580575</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="9">
         <v>48</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="10">
         <v>2503201001312</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E51" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F51" s="13"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E51" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="F51" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G51" s="21"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="9">
         <v>49</v>
       </c>
-      <c r="B52" s="11">
+      <c r="B52" s="10">
         <v>2503201001315</v>
       </c>
-      <c r="C52" s="11" t="s">
+      <c r="C52" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="D52" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E52" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F52" s="13"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E52" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F52" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G52" s="10">
+        <v>7290979690</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="9">
         <v>50</v>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="10">
         <v>2503201001318</v>
       </c>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="D53" s="10" t="s">
+      <c r="D53" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E53" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F53" s="13"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E53" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="F53" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G53" s="21"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="9">
         <v>51</v>
       </c>
-      <c r="B54" s="11">
+      <c r="B54" s="10">
         <v>2503201001323</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="D54" s="10" t="s">
+      <c r="D54" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="E54" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F54" s="13"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E54" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G54" s="21"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="9">
         <v>52</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="10">
         <v>2503201001328</v>
       </c>
-      <c r="C55" s="11" t="s">
+      <c r="C55" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="D55" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="E55" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F55" s="13"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E55" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G55" s="21"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="9">
         <v>53</v>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="10">
         <v>2503201001329</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D56" s="10" t="s">
+      <c r="D56" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="E56" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F56" s="13"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E56" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="F56" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G56" s="10">
+        <v>9216991969</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="9">
         <v>54</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="10">
         <v>2503201001331</v>
       </c>
-      <c r="C57" s="11" t="s">
+      <c r="C57" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="D57" s="10" t="s">
+      <c r="D57" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="E57" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F57" s="13"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E57" s="18" t="s">
+        <v>387</v>
+      </c>
+      <c r="F57" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G57" s="21"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="9">
         <v>55</v>
       </c>
-      <c r="B58" s="11">
+      <c r="B58" s="10">
         <v>2503201001334</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="D58" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="E58" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F58" s="13"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E58" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="F58" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" s="10">
+        <v>9368172639</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="9">
         <v>56</v>
       </c>
-      <c r="B59" s="11">
+      <c r="B59" s="10">
         <v>2503201001337</v>
       </c>
-      <c r="C59" s="11" t="s">
+      <c r="C59" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D59" s="10" t="s">
+      <c r="D59" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="E59" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F59" s="13"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E59" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="F59" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G59" s="10">
+        <v>9759230430</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="9">
         <v>57</v>
       </c>
-      <c r="B60" s="11">
+      <c r="B60" s="10">
         <v>2503201001339</v>
       </c>
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D60" s="10" t="s">
+      <c r="D60" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E60" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F60" s="13"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E60" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="F60" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G60" s="10">
+        <v>9468218940</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="9">
         <v>58</v>
       </c>
-      <c r="B61" s="11">
+      <c r="B61" s="10">
         <v>2503201001348</v>
       </c>
-      <c r="C61" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="D61" s="10" t="s">
+      <c r="C61" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="D61" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="E61" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F61" s="13"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E61" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="F61" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G61" s="21"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="9">
         <v>59</v>
       </c>
-      <c r="B62" s="11">
+      <c r="B62" s="10">
         <v>2503201001349</v>
       </c>
-      <c r="C62" s="11" t="s">
+      <c r="C62" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="E62" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F62" s="13"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E62" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="F62" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G62" s="10">
+        <v>9359644186</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="9">
         <v>60</v>
       </c>
-      <c r="B63" s="11">
+      <c r="B63" s="10">
         <v>2503201001350</v>
       </c>
-      <c r="C63" s="11" t="s">
+      <c r="C63" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D63" s="10" t="s">
+      <c r="D63" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="E63" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F63" s="13"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E63" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="F63" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G63" s="10">
+        <v>9569223522</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="9">
         <v>61</v>
       </c>
-      <c r="B64" s="11">
+      <c r="B64" s="10">
         <v>2503201001351</v>
       </c>
-      <c r="C64" s="11" t="s">
+      <c r="C64" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="D64" s="10" t="s">
+      <c r="D64" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="E64" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F64" s="13"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E64" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="F64" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G64" s="10">
+        <v>9711497241</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="9">
         <v>62</v>
       </c>
-      <c r="B65" s="11">
+      <c r="B65" s="10">
         <v>2503201001353</v>
       </c>
-      <c r="C65" s="11" t="s">
+      <c r="C65" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D65" s="10" t="s">
+      <c r="D65" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="E65" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F65" s="13"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E65" s="18" t="s">
+        <v>395</v>
+      </c>
+      <c r="F65" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G65" s="10">
+        <v>9568174212</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="9">
         <v>63</v>
       </c>
-      <c r="B66" s="11">
+      <c r="B66" s="10">
         <v>2503201001355</v>
       </c>
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="E66" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F66" s="13"/>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E66" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="F66" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G66" s="21"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="9">
         <v>64</v>
       </c>
-      <c r="B67" s="11">
+      <c r="B67" s="10">
         <v>2503201001356</v>
       </c>
-      <c r="C67" s="11" t="s">
+      <c r="C67" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D67" s="10" t="s">
+      <c r="D67" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E67" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F67" s="13"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E67" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="F67" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G67" s="21"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="9">
         <v>65</v>
       </c>
-      <c r="B68" s="11">
+      <c r="B68" s="10">
         <v>2503201001360</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C68" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D68" s="10" t="s">
+      <c r="D68" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="E68" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F68" s="13"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E68" s="18" t="s">
+        <v>398</v>
+      </c>
+      <c r="F68" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G68" s="21"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="9">
         <v>66</v>
       </c>
-      <c r="B69" s="11">
+      <c r="B69" s="10">
         <v>2503201001361</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="D69" s="10" t="s">
+      <c r="D69" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="E69" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F69" s="13"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E69" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="F69" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G69" s="10">
+        <v>8630294638</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="9">
         <v>67</v>
       </c>
-      <c r="B70" s="11">
+      <c r="B70" s="10">
         <v>2503201001364</v>
       </c>
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="D70" s="10" t="s">
+      <c r="D70" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="E70" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F70" s="13"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E70" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="F70" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G70" s="21"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="9">
         <v>68</v>
       </c>
-      <c r="B71" s="12">
+      <c r="B71" s="11">
         <v>2503201001171</v>
       </c>
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="D71" s="8" t="s">
+      <c r="D71" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="E71" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F71" s="7">
+      <c r="E71" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="F71" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G71" s="20">
         <v>7268044873</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="9">
         <v>69</v>
       </c>
-      <c r="B72" s="12">
+      <c r="B72" s="11">
         <v>2503201001172</v>
       </c>
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D72" s="8" t="s">
+      <c r="D72" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="E72" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F72" s="7">
+      <c r="E72" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="F72" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G72" s="7">
         <v>7903267072</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="9">
         <v>70</v>
       </c>
-      <c r="B73" s="12">
+      <c r="B73" s="11">
         <v>2503201001174</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D73" s="8" t="s">
+      <c r="D73" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="E73" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F73" s="8"/>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E73" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="F73" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G73" s="8"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="9">
         <v>71</v>
       </c>
-      <c r="B74" s="12">
+      <c r="B74" s="11">
         <v>2503201001178</v>
       </c>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="D74" s="8" t="s">
+      <c r="D74" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="E74" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F74" s="8"/>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E74" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="F74" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G74" s="8"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="9">
         <v>72</v>
       </c>
-      <c r="B75" s="12">
+      <c r="B75" s="11">
         <v>2503201001179</v>
       </c>
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="D75" s="8" t="s">
+      <c r="D75" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="E75" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F75" s="8"/>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E75" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="F75" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G75" s="8"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="9">
         <v>73</v>
       </c>
-      <c r="B76" s="12">
+      <c r="B76" s="11">
         <v>2503201001180</v>
       </c>
-      <c r="C76" s="11" t="s">
+      <c r="C76" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="D76" s="8" t="s">
+      <c r="D76" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="E76" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F76" s="8"/>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E76" s="18" t="s">
+        <v>276</v>
+      </c>
+      <c r="F76" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G76" s="8"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="9">
         <v>74</v>
       </c>
-      <c r="B77" s="12">
+      <c r="B77" s="11">
         <v>2503201001181</v>
       </c>
-      <c r="C77" s="11" t="s">
+      <c r="C77" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D77" s="8" t="s">
+      <c r="D77" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="E77" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F77" s="8"/>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E77" s="18" t="s">
+        <v>277</v>
+      </c>
+      <c r="F77" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G77" s="8"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="9">
         <v>75</v>
       </c>
-      <c r="B78" s="12">
+      <c r="B78" s="11">
         <v>2503201001187</v>
       </c>
-      <c r="C78" s="11" t="s">
+      <c r="C78" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="D78" s="8" t="s">
+      <c r="D78" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="E78" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F78" s="8"/>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E78" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G78" s="8"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="9">
         <v>76</v>
       </c>
-      <c r="B79" s="12">
+      <c r="B79" s="11">
         <v>2503201001189</v>
       </c>
-      <c r="C79" s="11" t="s">
+      <c r="C79" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="D79" s="8" t="s">
+      <c r="D79" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="E79" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F79" s="8"/>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E79" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="F79" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G79" s="8"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="9">
         <v>77</v>
       </c>
-      <c r="B80" s="12">
+      <c r="B80" s="11">
         <v>2503201001194</v>
       </c>
-      <c r="C80" s="11" t="s">
+      <c r="C80" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="D80" s="8" t="s">
+      <c r="D80" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="E80" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F80" s="8"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E80" s="18" t="s">
+        <v>279</v>
+      </c>
+      <c r="F80" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G80" s="8"/>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="9">
         <v>78</v>
       </c>
-      <c r="B81" s="12">
+      <c r="B81" s="11">
         <v>2503201001198</v>
       </c>
       <c r="C81" s="7"/>
-      <c r="D81" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="E81" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F81" s="8"/>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D81" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="E81" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="F81" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G81" s="8"/>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="9">
         <v>79</v>
       </c>
-      <c r="B82" s="12">
+      <c r="B82" s="11">
         <v>2503201001204</v>
       </c>
-      <c r="C82" s="11" t="s">
+      <c r="C82" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="D82" s="8" t="s">
+      <c r="D82" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="E82" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F82" s="8"/>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E82" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="F82" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G82" s="8"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="9">
         <v>80</v>
       </c>
-      <c r="B83" s="12">
+      <c r="B83" s="11">
         <v>2503201001205</v>
       </c>
-      <c r="C83" s="11" t="s">
+      <c r="C83" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="D83" s="8" t="s">
+      <c r="D83" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="E83" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F83" s="8"/>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E83" s="18" t="s">
+        <v>282</v>
+      </c>
+      <c r="F83" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G83" s="8"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="9">
         <v>81</v>
       </c>
-      <c r="B84" s="12">
+      <c r="B84" s="11">
         <v>2503201001210</v>
       </c>
-      <c r="C84" s="11" t="s">
+      <c r="C84" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="D84" s="8" t="s">
+      <c r="D84" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="E84" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F84" s="8"/>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E84" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="F84" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G84" s="8"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="9">
         <v>82</v>
       </c>
-      <c r="B85" s="12">
+      <c r="B85" s="11">
         <v>2503201001213</v>
       </c>
-      <c r="C85" s="11" t="s">
+      <c r="C85" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="D85" s="8" t="s">
+      <c r="D85" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="E85" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F85" s="7">
+      <c r="E85" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="F85" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G85" s="7">
         <v>7978764290</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="9">
         <v>83</v>
       </c>
-      <c r="B86" s="12">
+      <c r="B86" s="11">
         <v>2503201001222</v>
       </c>
-      <c r="C86" s="11" t="s">
+      <c r="C86" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="D86" s="8" t="s">
+      <c r="D86" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="E86" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F86" s="8"/>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E86" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="F86" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G86" s="8"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="9">
         <v>84</v>
       </c>
-      <c r="B87" s="12">
+      <c r="B87" s="11">
         <v>2503201001226</v>
       </c>
-      <c r="C87" s="11" t="s">
+      <c r="C87" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="D87" s="8" t="s">
+      <c r="D87" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="E87" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F87" s="7">
+      <c r="E87" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="F87" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G87" s="7">
         <v>8445220989</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="9">
         <v>85</v>
       </c>
-      <c r="B88" s="12">
+      <c r="B88" s="11">
         <v>2503201001229</v>
       </c>
-      <c r="C88" s="11" t="s">
+      <c r="C88" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="D88" s="8" t="s">
+      <c r="D88" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="E88" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F88" s="8"/>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E88" s="18" t="s">
+        <v>287</v>
+      </c>
+      <c r="F88" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G88" s="8"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="9">
         <v>86</v>
       </c>
-      <c r="B89" s="12">
+      <c r="B89" s="11">
         <v>2503201001231</v>
       </c>
-      <c r="C89" s="11" t="s">
+      <c r="C89" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="D89" s="8" t="s">
+      <c r="D89" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="E89" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F89" s="8"/>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E89" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="F89" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G89" s="8"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="9">
         <v>87</v>
       </c>
-      <c r="B90" s="12">
+      <c r="B90" s="11">
         <v>2503201001237</v>
       </c>
-      <c r="C90" s="11" t="s">
+      <c r="C90" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="D90" s="8" t="s">
+      <c r="D90" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E90" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F90" s="7">
+      <c r="E90" s="18" t="s">
+        <v>289</v>
+      </c>
+      <c r="F90" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G90" s="7">
         <v>9286323915</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="9">
         <v>88</v>
       </c>
-      <c r="B91" s="12">
+      <c r="B91" s="11">
         <v>2503201001240</v>
       </c>
-      <c r="C91" s="11" t="s">
+      <c r="C91" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="D91" s="8" t="s">
+      <c r="D91" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="E91" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F91" s="8"/>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E91" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="F91" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G91" s="8"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="9">
         <v>89</v>
       </c>
-      <c r="B92" s="12">
+      <c r="B92" s="11">
         <v>2503201001241</v>
       </c>
-      <c r="C92" s="11" t="s">
+      <c r="C92" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="D92" s="8" t="s">
+      <c r="D92" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="E92" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F92" s="8"/>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E92" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="F92" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G92" s="8"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" s="9">
         <v>90</v>
       </c>
-      <c r="B93" s="12">
+      <c r="B93" s="11">
         <v>2503201001242</v>
       </c>
-      <c r="C93" s="11" t="s">
+      <c r="C93" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="D93" s="8" t="s">
+      <c r="D93" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="E93" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F93" s="8"/>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E93" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="F93" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G93" s="8"/>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="9">
         <v>91</v>
       </c>
-      <c r="B94" s="12">
+      <c r="B94" s="11">
         <v>2503201001243</v>
       </c>
-      <c r="C94" s="11" t="s">
+      <c r="C94" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="D94" s="8" t="s">
+      <c r="D94" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="E94" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F94" s="8"/>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E94" s="18" t="s">
+        <v>293</v>
+      </c>
+      <c r="F94" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G94" s="8"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="9">
         <v>92</v>
       </c>
-      <c r="B95" s="12">
+      <c r="B95" s="11">
         <v>2503201001244</v>
       </c>
-      <c r="C95" s="11" t="s">
+      <c r="C95" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="D95" s="8" t="s">
+      <c r="D95" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="E95" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F95" s="8"/>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E95" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="F95" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G95" s="8"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="9">
         <v>93</v>
       </c>
-      <c r="B96" s="12">
+      <c r="B96" s="11">
         <v>2503201001245</v>
       </c>
-      <c r="C96" s="11" t="s">
+      <c r="C96" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="D96" s="8" t="s">
+      <c r="D96" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="E96" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F96" s="7">
+      <c r="E96" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="F96" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G96" s="7">
         <v>9625340387</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="9">
         <v>94</v>
       </c>
-      <c r="B97" s="12">
+      <c r="B97" s="11">
         <v>2503201001246</v>
       </c>
-      <c r="C97" s="11" t="s">
+      <c r="C97" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="D97" s="8" t="s">
+      <c r="D97" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="E97" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F97" s="8"/>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E97" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="F97" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G97" s="8"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" s="9">
         <v>95</v>
       </c>
-      <c r="B98" s="12">
+      <c r="B98" s="11">
         <v>2503201001247</v>
       </c>
-      <c r="C98" s="11" t="s">
+      <c r="C98" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="D98" s="8" t="s">
+      <c r="D98" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="E98" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F98" s="8"/>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E98" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="F98" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G98" s="8"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="9">
         <v>96</v>
       </c>
-      <c r="B99" s="12">
+      <c r="B99" s="11">
         <v>2503201001248</v>
       </c>
-      <c r="C99" s="11" t="s">
+      <c r="C99" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D99" s="8" t="s">
+      <c r="D99" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="E99" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F99" s="8"/>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E99" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="F99" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G99" s="8"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" s="9">
         <v>97</v>
       </c>
-      <c r="B100" s="12">
+      <c r="B100" s="11">
         <v>2503201001251</v>
       </c>
-      <c r="C100" s="11" t="s">
+      <c r="C100" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="D100" s="8" t="s">
+      <c r="D100" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="E100" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F100" s="7">
+      <c r="E100" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="F100" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G100" s="7">
         <v>8576094319</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="9">
         <v>98</v>
       </c>
-      <c r="B101" s="12">
+      <c r="B101" s="11">
         <v>2503201001254</v>
       </c>
-      <c r="C101" s="11" t="s">
+      <c r="C101" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="D101" s="8" t="s">
+      <c r="D101" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="E101" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F101" s="8"/>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E101" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="F101" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G101" s="8"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" s="9">
         <v>99</v>
       </c>
-      <c r="B102" s="12">
+      <c r="B102" s="11">
         <v>2503201001255</v>
       </c>
-      <c r="C102" s="11" t="s">
+      <c r="C102" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="D102" s="8" t="s">
+      <c r="D102" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="E102" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F102" s="7">
+      <c r="E102" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="F102" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G102" s="7">
         <v>7817924108</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="9">
         <v>100</v>
       </c>
-      <c r="B103" s="12">
+      <c r="B103" s="11">
         <v>2503201001258</v>
       </c>
-      <c r="C103" s="11" t="s">
+      <c r="C103" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="D103" s="8" t="s">
+      <c r="D103" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="E103" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F103" s="8"/>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E103" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="F103" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G103" s="8"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="9">
         <v>101</v>
       </c>
-      <c r="B104" s="12">
+      <c r="B104" s="11">
         <v>2503201001259</v>
       </c>
-      <c r="C104" s="11" t="s">
+      <c r="C104" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="D104" s="8" t="s">
+      <c r="D104" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E104" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F104" s="7">
+      <c r="E104" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="F104" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G104" s="7">
         <v>8189054212</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" s="9">
         <v>102</v>
       </c>
-      <c r="B105" s="12">
+      <c r="B105" s="11">
         <v>2503201001263</v>
       </c>
-      <c r="C105" s="11" t="s">
+      <c r="C105" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="D105" s="8" t="s">
+      <c r="D105" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="E105" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F105" s="7">
+      <c r="E105" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="F105" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G105" s="7">
         <v>7355524407</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="9">
         <v>103</v>
       </c>
-      <c r="B106" s="12">
+      <c r="B106" s="11">
         <v>2503201001265</v>
       </c>
-      <c r="C106" s="11" t="s">
+      <c r="C106" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="D106" s="8" t="s">
+      <c r="D106" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="E106" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F106" s="8"/>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E106" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="F106" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G106" s="8"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" s="9">
         <v>104</v>
       </c>
-      <c r="B107" s="12">
+      <c r="B107" s="11">
         <v>2503201001272</v>
       </c>
-      <c r="C107" s="11" t="s">
+      <c r="C107" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="D107" s="8" t="s">
+      <c r="D107" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="E107" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F107" s="8"/>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E107" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="F107" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G107" s="8"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108" s="9">
         <v>105</v>
       </c>
-      <c r="B108" s="12">
+      <c r="B108" s="11">
         <v>2503201001276</v>
       </c>
-      <c r="C108" s="11" t="s">
+      <c r="C108" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="D108" s="8" t="s">
+      <c r="D108" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="E108" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F108" s="7">
+      <c r="E108" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="F108" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G108" s="7">
         <v>9140244464</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109" s="9">
         <v>106</v>
       </c>
-      <c r="B109" s="12">
+      <c r="B109" s="11">
         <v>2503201001277</v>
       </c>
-      <c r="C109" s="11" t="s">
+      <c r="C109" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="D109" s="8" t="s">
+      <c r="D109" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="E109" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F109" s="8"/>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E109" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="F109" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G109" s="8"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="9">
         <v>107</v>
       </c>
-      <c r="B110" s="12">
+      <c r="B110" s="11">
         <v>2503201001280</v>
       </c>
-      <c r="C110" s="11" t="s">
+      <c r="C110" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="D110" s="8" t="s">
+      <c r="D110" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="E110" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F110" s="8"/>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E110" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="F110" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G110" s="8"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" s="9">
         <v>108</v>
       </c>
-      <c r="B111" s="12">
+      <c r="B111" s="11">
         <v>2503201001281</v>
       </c>
-      <c r="C111" s="11" t="s">
+      <c r="C111" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="D111" s="8" t="s">
+      <c r="D111" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="E111" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F111" s="7">
+      <c r="E111" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="F111" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G111" s="7">
         <v>9318487216</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" s="9">
         <v>109</v>
       </c>
-      <c r="B112" s="12">
+      <c r="B112" s="11">
         <v>2503201001285</v>
       </c>
-      <c r="C112" s="11" t="s">
+      <c r="C112" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="D112" s="8" t="s">
+      <c r="D112" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="E112" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F112" s="7">
+      <c r="E112" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="F112" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G112" s="7">
         <v>7983220964</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A113" s="9">
         <v>110</v>
       </c>
-      <c r="B113" s="12">
+      <c r="B113" s="11">
         <v>2503201001287</v>
       </c>
-      <c r="C113" s="11" t="s">
+      <c r="C113" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="D113" s="8" t="s">
+      <c r="D113" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="E113" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F113" s="8"/>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E113" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="F113" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G113" s="8"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114" s="9">
         <v>111</v>
       </c>
-      <c r="B114" s="12">
+      <c r="B114" s="11">
         <v>2503201001289</v>
       </c>
-      <c r="C114" s="11" t="s">
+      <c r="C114" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="D114" s="8" t="s">
+      <c r="D114" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E114" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F114" s="7">
+      <c r="E114" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="F114" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G114" s="7">
         <v>9012562896</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115" s="9">
         <v>112</v>
       </c>
-      <c r="B115" s="12">
+      <c r="B115" s="11">
         <v>2503201001294</v>
       </c>
-      <c r="C115" s="11" t="s">
+      <c r="C115" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="D115" s="8" t="s">
+      <c r="D115" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="E115" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F115" s="7">
+      <c r="E115" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="F115" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G115" s="7">
         <v>8194020000</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116" s="9">
         <v>113</v>
       </c>
-      <c r="B116" s="12">
+      <c r="B116" s="11">
         <v>2503201001299</v>
       </c>
-      <c r="C116" s="11" t="s">
+      <c r="C116" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="D116" s="8" t="s">
+      <c r="D116" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="E116" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F116" s="8"/>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E116" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="F116" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G116" s="8"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117" s="9">
         <v>114</v>
       </c>
-      <c r="B117" s="12">
+      <c r="B117" s="11">
         <v>2503201001302</v>
       </c>
-      <c r="C117" s="11" t="s">
+      <c r="C117" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="D117" s="8" t="s">
+      <c r="D117" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="E117" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F117" s="7">
+      <c r="E117" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="F117" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G117" s="7">
         <v>9310703932</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118" s="9">
         <v>115</v>
       </c>
-      <c r="B118" s="12">
+      <c r="B118" s="11">
         <v>2503201001303</v>
       </c>
-      <c r="C118" s="11" t="s">
+      <c r="C118" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="D118" s="8" t="s">
+      <c r="D118" s="14" t="s">
         <v>226</v>
       </c>
-      <c r="E118" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F118" s="7">
+      <c r="E118" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="F118" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G118" s="7">
         <v>9205003696</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119" s="9">
         <v>116</v>
       </c>
-      <c r="B119" s="12">
+      <c r="B119" s="11">
         <v>2503201001313</v>
       </c>
-      <c r="C119" s="11" t="s">
+      <c r="C119" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="D119" s="8" t="s">
+      <c r="D119" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="E119" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F119" s="7">
+      <c r="E119" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F119" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G119" s="7">
         <v>7452082079</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120" s="9">
         <v>117</v>
       </c>
-      <c r="B120" s="12">
+      <c r="B120" s="11">
         <v>2503201001314</v>
       </c>
-      <c r="C120" s="11" t="s">
+      <c r="C120" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="D120" s="8" t="s">
+      <c r="D120" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="E120" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F120" s="8"/>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E120" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="F120" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G120" s="8"/>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" s="9">
         <v>118</v>
       </c>
-      <c r="B121" s="12">
+      <c r="B121" s="11">
         <v>2503201001316</v>
       </c>
-      <c r="C121" s="11" t="s">
+      <c r="C121" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="D121" s="8" t="s">
+      <c r="D121" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="E121" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F121" s="7">
+      <c r="E121" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="F121" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G121" s="7">
         <v>7380535080</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122" s="9">
         <v>119</v>
       </c>
-      <c r="B122" s="12">
+      <c r="B122" s="11">
         <v>2503201001319</v>
       </c>
-      <c r="C122" s="11" t="s">
+      <c r="C122" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="D122" s="8" t="s">
+      <c r="D122" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="E122" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F122" s="7">
+      <c r="E122" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F122" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G122" s="7">
         <v>9984457250</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123" s="9">
         <v>120</v>
       </c>
-      <c r="B123" s="12">
+      <c r="B123" s="11">
         <v>2503201001321</v>
       </c>
-      <c r="C123" s="11" t="s">
+      <c r="C123" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="D123" s="8" t="s">
+      <c r="D123" s="14" t="s">
         <v>236</v>
       </c>
-      <c r="E123" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F123" s="8"/>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E123" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="F123" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G123" s="8"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124" s="9">
         <v>121</v>
       </c>
-      <c r="B124" s="12">
+      <c r="B124" s="11">
         <v>2503201001322</v>
       </c>
-      <c r="C124" s="11" t="s">
+      <c r="C124" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="D124" s="8" t="s">
+      <c r="D124" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="E124" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F124" s="8"/>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E124" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F124" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G124" s="8"/>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125" s="9">
         <v>122</v>
       </c>
-      <c r="B125" s="12">
+      <c r="B125" s="11">
         <v>2503201001324</v>
       </c>
-      <c r="C125" s="11" t="s">
+      <c r="C125" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="D125" s="8" t="s">
+      <c r="D125" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="E125" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F125" s="8"/>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E125" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="F125" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G125" s="8"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126" s="9">
         <v>123</v>
       </c>
-      <c r="B126" s="12">
+      <c r="B126" s="11">
         <v>2503201001332</v>
       </c>
-      <c r="C126" s="11" t="s">
+      <c r="C126" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="D126" s="8" t="s">
+      <c r="D126" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="E126" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F126" s="8"/>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E126" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="F126" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G126" s="8"/>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127" s="9">
         <v>124</v>
       </c>
-      <c r="B127" s="12">
+      <c r="B127" s="11">
         <v>2503201001333</v>
       </c>
-      <c r="C127" s="11" t="s">
+      <c r="C127" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="D127" s="8" t="s">
+      <c r="D127" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="E127" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F127" s="8"/>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E127" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="F127" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G127" s="8"/>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128" s="9">
         <v>125</v>
       </c>
-      <c r="B128" s="12">
+      <c r="B128" s="11">
         <v>2503201001336</v>
       </c>
-      <c r="C128" s="11" t="s">
+      <c r="C128" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="D128" s="8" t="s">
+      <c r="D128" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="E128" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F128" s="8"/>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E128" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="F128" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G128" s="8"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129" s="9">
         <v>126</v>
       </c>
-      <c r="B129" s="12">
+      <c r="B129" s="11">
         <v>2503201001342</v>
       </c>
-      <c r="C129" s="11" t="s">
+      <c r="C129" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="D129" s="8" t="s">
+      <c r="D129" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="E129" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F129" s="8"/>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E129" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="F129" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G129" s="8"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130" s="9">
         <v>127</v>
       </c>
-      <c r="B130" s="12">
+      <c r="B130" s="11">
         <v>2503201001343</v>
       </c>
-      <c r="C130" s="11" t="s">
+      <c r="C130" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="D130" s="8" t="s">
+      <c r="D130" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="E130" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F130" s="8"/>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E130" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="F130" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G130" s="8"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131" s="9">
         <v>128</v>
       </c>
-      <c r="B131" s="12">
+      <c r="B131" s="11">
         <v>2503201001344</v>
       </c>
-      <c r="C131" s="11" t="s">
+      <c r="C131" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="D131" s="8" t="s">
+      <c r="D131" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="E131" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F131" s="8"/>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E131" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="F131" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G131" s="8"/>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132" s="9">
         <v>129</v>
       </c>
-      <c r="B132" s="12">
+      <c r="B132" s="11">
         <v>2503201001347</v>
       </c>
-      <c r="C132" s="11" t="s">
+      <c r="C132" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="D132" s="8" t="s">
+      <c r="D132" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="E132" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F132" s="8"/>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E132" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="F132" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G132" s="8"/>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133" s="9">
         <v>130</v>
       </c>
-      <c r="B133" s="12">
+      <c r="B133" s="11">
         <v>2503201001352</v>
       </c>
-      <c r="C133" s="11" t="s">
+      <c r="C133" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="D133" s="8" t="s">
+      <c r="D133" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="E133" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F133" s="7">
+      <c r="E133" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="F133" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G133" s="7">
         <v>8795129372</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A134" s="9">
         <v>131</v>
       </c>
-      <c r="B134" s="12">
+      <c r="B134" s="11">
         <v>2503201001354</v>
       </c>
-      <c r="C134" s="11" t="s">
+      <c r="C134" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="D134" s="8" t="s">
+      <c r="D134" s="14" t="s">
         <v>254</v>
       </c>
-      <c r="E134" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F134" s="7">
+      <c r="E134" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="F134" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G134" s="7">
         <v>9289512902</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A135" s="9">
         <v>132</v>
       </c>
-      <c r="B135" s="12">
+      <c r="B135" s="11">
         <v>2503201001357</v>
       </c>
-      <c r="C135" s="11" t="s">
+      <c r="C135" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="D135" s="8" t="s">
+      <c r="D135" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="E135" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F135" s="8"/>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E135" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="F135" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G135" s="8"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136" s="9">
         <v>133</v>
       </c>
-      <c r="B136" s="12">
+      <c r="B136" s="11">
         <v>2503201001367</v>
       </c>
-      <c r="C136" s="11" t="s">
+      <c r="C136" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="D136" s="8" t="s">
+      <c r="D136" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="E136" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F136" s="8"/>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E136" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="F136" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G136" s="8"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A137" s="9">
         <v>134</v>
       </c>
-      <c r="B137" s="14">
+      <c r="B137" s="12">
         <v>2503201001368</v>
       </c>
-      <c r="C137" s="11" t="s">
+      <c r="C137" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="D137" s="8" t="s">
+      <c r="D137" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="E137" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="F137" s="8"/>
+      <c r="E137" s="18" t="s">
+        <v>335</v>
+      </c>
+      <c r="F137" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G137" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>